<commit_message>
train model for 2025 beers
</commit_message>
<xml_diff>
--- a/backend/Statistikk Juleøl.xlsx
+++ b/backend/Statistikk Juleøl.xlsx
@@ -7,25 +7,26 @@
     <sheet state="visible" name="2022" sheetId="2" r:id="rId5"/>
     <sheet state="visible" name="2023" sheetId="3" r:id="rId6"/>
     <sheet state="visible" name="2024" sheetId="4" r:id="rId7"/>
+    <sheet state="visible" name="2025" sheetId="5" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="1" name="Z_C71C843A_EAB5_42B1_B1FD_81E558391A10_.wvu.FilterData">'2022'!$A$1:$A$14</definedName>
-    <definedName hidden="1" localSheetId="2" name="Z_C71C843A_EAB5_42B1_B1FD_81E558391A10_.wvu.FilterData">'2023'!$A$1:$A$14</definedName>
-    <definedName hidden="1" localSheetId="0" name="Z_A5D866E3_0697_42C0_A55F_3D9EB20CFB23_.wvu.FilterData">'2020'!$J$1:$J$19</definedName>
-    <definedName hidden="1" localSheetId="1" name="Z_A5D866E3_0697_42C0_A55F_3D9EB20CFB23_.wvu.FilterData">'2022'!$A$2:$J$14</definedName>
-    <definedName hidden="1" localSheetId="2" name="Z_A5D866E3_0697_42C0_A55F_3D9EB20CFB23_.wvu.FilterData">'2023'!$A$2:$J$14</definedName>
-    <definedName hidden="1" localSheetId="3" name="Z_A5D866E3_0697_42C0_A55F_3D9EB20CFB23_.wvu.FilterData">'2024'!$B$2:$I$30</definedName>
+    <definedName hidden="1" localSheetId="1" name="Z_6393740B_0DC1_4FF3_81AB_78517B923F87_.wvu.FilterData">'2022'!$A$1:$A$14</definedName>
+    <definedName hidden="1" localSheetId="2" name="Z_6393740B_0DC1_4FF3_81AB_78517B923F87_.wvu.FilterData">'2023'!$A$1:$A$14</definedName>
+    <definedName hidden="1" localSheetId="0" name="Z_BE750BA2_1E5A_4896_A3E0_39DCEBB13DE6_.wvu.FilterData">'2020'!$J$1:$J$19</definedName>
+    <definedName hidden="1" localSheetId="1" name="Z_BE750BA2_1E5A_4896_A3E0_39DCEBB13DE6_.wvu.FilterData">'2022'!$A$2:$J$14</definedName>
+    <definedName hidden="1" localSheetId="2" name="Z_BE750BA2_1E5A_4896_A3E0_39DCEBB13DE6_.wvu.FilterData">'2023'!$A$2:$J$14</definedName>
+    <definedName hidden="1" localSheetId="3" name="Z_BE750BA2_1E5A_4896_A3E0_39DCEBB13DE6_.wvu.FilterData">'2024'!$B$2:$I$30</definedName>
   </definedNames>
   <calcPr/>
   <customWorkbookViews>
-    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{C71C843A-EAB5-42B1-B1FD-81E558391A10}" name="Filter 2"/>
-    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{A5D866E3-0697-42C0-A55F-3D9EB20CFB23}" name="Filter 1"/>
+    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{6393740B-0DC1-4FF3-81AB-78517B923F87}" name="Filter 2"/>
+    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{BE750BA2-1E5A-4896-A3E0-39DCEBB13DE6}" name="Filter 1"/>
   </customWorkbookViews>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="117">
   <si>
     <t>Nummer</t>
   </si>
@@ -138,9 +139,6 @@
     <t>Mack Juleøl</t>
   </si>
   <si>
-    <t>Macks Ølbryggeri</t>
-  </si>
-  <si>
     <t>Nordlandspils Juleøl</t>
   </si>
   <si>
@@ -193,6 +191,9 @@
   </si>
   <si>
     <t>IPA</t>
+  </si>
+  <si>
+    <t>Macks Ølbryggeri</t>
   </si>
   <si>
     <t>Gouden Carolus Christmas</t>
@@ -338,6 +339,45 @@
   <si>
     <t>Hansa Juleøl</t>
   </si>
+  <si>
+    <t>Flåklypa Spesial Juleøl</t>
+  </si>
+  <si>
+    <t>Nøisom</t>
+  </si>
+  <si>
+    <t>To Øl Jule Sovs Hazy IPA</t>
+  </si>
+  <si>
+    <t>Nøgne Ø Julequad</t>
+  </si>
+  <si>
+    <t>Ringnes Juleøl Sterk</t>
+  </si>
+  <si>
+    <t>Delirium</t>
+  </si>
+  <si>
+    <t>Cervisiam Santa Mental Sour Cream Pie</t>
+  </si>
+  <si>
+    <t>Cervisiam Bryggeri</t>
+  </si>
+  <si>
+    <t>Julekula 2025 Barrel Aged</t>
+  </si>
+  <si>
+    <t>Tuborg Juleøl Butikk</t>
+  </si>
+  <si>
+    <t>Gildeskål Saison</t>
+  </si>
+  <si>
+    <t>Bådin</t>
+  </si>
+  <si>
+    <t>Santas Break Red Lager</t>
+  </si>
 </sst>
 </file>
 
@@ -378,7 +418,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -427,6 +467,15 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -448,6 +497,10 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -1000,7 +1053,7 @@
         <v>36</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>27</v>
@@ -1027,10 +1080,10 @@
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="3"/>
       <c r="B13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>27</v>
@@ -1057,10 +1110,10 @@
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="3"/>
       <c r="B14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>27</v>
@@ -1087,13 +1140,13 @@
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="3"/>
       <c r="B15" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="8" t="s">
         <v>43</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>44</v>
       </c>
       <c r="E15" s="4">
         <v>0.06</v>
@@ -1117,10 +1170,10 @@
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="3"/>
       <c r="B16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>27</v>
@@ -1147,7 +1200,7 @@
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="3"/>
       <c r="B17" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>19</v>
@@ -1177,10 +1230,10 @@
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="3"/>
       <c r="B18" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>27</v>
@@ -1207,10 +1260,10 @@
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="3"/>
       <c r="B19" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>27</v>
@@ -1238,7 +1291,7 @@
     <row r="21" ht="15.75" customHeight="1"/>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{A5D866E3-0697-42C0-A55F-3D9EB20CFB23}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{BE750BA2-1E5A-4896-A3E0-39DCEBB13DE6}" filter="1" showAutoFilter="1">
       <autoFilter ref="$J$1:$J$19"/>
     </customSheetView>
   </customSheetViews>
@@ -1304,13 +1357,13 @@
         <v>11.0</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="E2" s="4">
         <v>0.06</v>
@@ -1338,13 +1391,13 @@
         <v>1.0</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="E3" s="4">
         <v>0.065</v>
@@ -1373,7 +1426,7 @@
         <v>36</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>27</v>
@@ -1608,10 +1661,10 @@
         <v>8.0</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>27</v>
@@ -9616,10 +9669,10 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{A5D866E3-0697-42C0-A55F-3D9EB20CFB23}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{BE750BA2-1E5A-4896-A3E0-39DCEBB13DE6}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$2:$J$14"/>
     </customSheetView>
-    <customSheetView guid="{C71C843A-EAB5-42B1-B1FD-81E558391A10}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{6393740B-0DC1-4FF3-81AB-78517B923F87}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$A$14">
         <filterColumn colId="0">
           <filters>
@@ -9701,13 +9754,13 @@
         <v>6.0</v>
       </c>
       <c r="B2" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>52</v>
       </c>
       <c r="E2" s="15">
         <v>0.06</v>
@@ -9776,7 +9829,7 @@
         <v>72</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>20</v>
@@ -9921,7 +9974,7 @@
         <v>16</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E8" s="15">
         <v>0.085</v>
@@ -9954,7 +10007,7 @@
         <v>36</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>27</v>
@@ -18021,10 +18074,10 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{A5D866E3-0697-42C0-A55F-3D9EB20CFB23}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{BE750BA2-1E5A-4896-A3E0-39DCEBB13DE6}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$2:$J$14"/>
     </customSheetView>
-    <customSheetView guid="{C71C843A-EAB5-42B1-B1FD-81E558391A10}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{6393740B-0DC1-4FF3-81AB-78517B923F87}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$A$14">
         <filterColumn colId="0">
           <filters>
@@ -18147,7 +18200,7 @@
         <v>84</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>20</v>
@@ -18339,13 +18392,13 @@
         <v>2.0</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="14" t="s">
         <v>51</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>52</v>
       </c>
       <c r="E8" s="15">
         <v>0.06</v>
@@ -18420,7 +18473,7 @@
         <v>93</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>20</v>
@@ -18501,7 +18554,7 @@
         <v>95</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E12" s="15">
         <v>0.074</v>
@@ -18579,7 +18632,7 @@
         <v>91</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E14" s="15">
         <v>0.06</v>
@@ -18618,7 +18671,7 @@
         <v>91</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E15" s="15">
         <v>0.065</v>
@@ -18654,7 +18707,7 @@
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>27</v>
@@ -18693,7 +18746,7 @@
         <v>100</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>27</v>
@@ -18732,7 +18785,7 @@
         <v>101</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>27</v>
@@ -18771,7 +18824,7 @@
         <v>102</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>27</v>
@@ -18846,10 +18899,10 @@
         <v>19.0</v>
       </c>
       <c r="B21" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>27</v>
@@ -24817,7 +24870,7 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{A5D866E3-0697-42C0-A55F-3D9EB20CFB23}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{BE750BA2-1E5A-4896-A3E0-39DCEBB13DE6}" filter="1" showAutoFilter="1">
       <autoFilter ref="$B$2:$I$30"/>
     </customSheetView>
   </customSheetViews>
@@ -24826,4 +24879,670 @@
   <pageSetup fitToHeight="0" paperSize="9" orientation="landscape" pageOrder="overThenDown"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <v>8.0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="20">
+        <v>0.06</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="G2" s="21">
+        <v>69.9</v>
+      </c>
+      <c r="H2" s="19">
+        <v>85.0</v>
+      </c>
+      <c r="I2" s="19">
+        <v>80.0</v>
+      </c>
+      <c r="J2" s="2">
+        <v>100.0</v>
+      </c>
+      <c r="K2" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="L2" s="22">
+        <f t="shared" ref="L2:L16" si="1">AVERAGE(H2:K2)</f>
+        <v>84.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" s="20">
+        <v>0.06</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="G3" s="21">
+        <v>159.9</v>
+      </c>
+      <c r="H3" s="19">
+        <v>87.0</v>
+      </c>
+      <c r="I3" s="19">
+        <v>75.0</v>
+      </c>
+      <c r="J3" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="K3" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="L3" s="22">
+        <f t="shared" si="1"/>
+        <v>75.75</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>9.0</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="20">
+        <v>0.102</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G4" s="21">
+        <v>138.0</v>
+      </c>
+      <c r="H4" s="19">
+        <v>74.0</v>
+      </c>
+      <c r="I4" s="19">
+        <v>67.0</v>
+      </c>
+      <c r="J4" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="K4" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="L4" s="22">
+        <f t="shared" si="1"/>
+        <v>68.25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>10.0</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" s="20">
+        <v>0.061</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.44</v>
+      </c>
+      <c r="G5" s="21">
+        <v>91.9</v>
+      </c>
+      <c r="H5" s="19">
+        <v>72.0</v>
+      </c>
+      <c r="I5" s="19">
+        <v>65.0</v>
+      </c>
+      <c r="J5" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="K5" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="L5" s="22">
+        <f t="shared" si="1"/>
+        <v>66.75</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>12.0</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="20">
+        <v>0.065</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="G6" s="2">
+        <v>49.9</v>
+      </c>
+      <c r="H6" s="19">
+        <v>82.0</v>
+      </c>
+      <c r="I6" s="19">
+        <v>60.0</v>
+      </c>
+      <c r="J6" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="K6" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="L6" s="22">
+        <f t="shared" si="1"/>
+        <v>66.75</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="20">
+        <v>0.09</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="G7" s="2">
+        <v>50.1</v>
+      </c>
+      <c r="H7" s="19">
+        <v>55.0</v>
+      </c>
+      <c r="I7" s="19">
+        <v>68.0</v>
+      </c>
+      <c r="J7" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="K7" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="L7" s="22">
+        <f t="shared" si="1"/>
+        <v>61.75</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>13.0</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" s="20">
+        <v>0.12</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G8" s="2">
+        <v>89.9</v>
+      </c>
+      <c r="H8" s="19">
+        <v>50.0</v>
+      </c>
+      <c r="I8" s="19">
+        <v>70.0</v>
+      </c>
+      <c r="J8" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="K8" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="L8" s="22">
+        <f t="shared" si="1"/>
+        <v>59.25</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="20">
+        <v>0.063</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="G9" s="21">
+        <v>41.9</v>
+      </c>
+      <c r="H9" s="19">
+        <v>65.0</v>
+      </c>
+      <c r="I9" s="19">
+        <v>50.0</v>
+      </c>
+      <c r="J9" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="K9" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="L9" s="22">
+        <f t="shared" si="1"/>
+        <v>58.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="20">
+        <v>0.06</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="G10" s="21">
+        <v>44.9</v>
+      </c>
+      <c r="H10" s="19">
+        <v>75.0</v>
+      </c>
+      <c r="I10" s="19">
+        <v>66.0</v>
+      </c>
+      <c r="J10" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="K10" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="L10" s="22">
+        <f t="shared" si="1"/>
+        <v>57.75</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2">
+        <v>7.0</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="20">
+        <v>0.1</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="G11" s="21">
+        <v>159.9</v>
+      </c>
+      <c r="H11" s="19">
+        <v>76.0</v>
+      </c>
+      <c r="I11" s="19">
+        <v>25.0</v>
+      </c>
+      <c r="J11" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="K11" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="L11" s="22">
+        <f t="shared" si="1"/>
+        <v>56.75</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="20">
+        <v>0.057</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="G12" s="21">
+        <v>90.4</v>
+      </c>
+      <c r="H12" s="19">
+        <v>55.0</v>
+      </c>
+      <c r="I12" s="19">
+        <v>69.0</v>
+      </c>
+      <c r="J12" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="K12" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="L12" s="22">
+        <f t="shared" si="1"/>
+        <v>56.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2">
+        <v>11.0</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="20">
+        <v>0.08</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.44</v>
+      </c>
+      <c r="G13" s="21">
+        <v>120.2</v>
+      </c>
+      <c r="H13" s="19">
+        <v>62.0</v>
+      </c>
+      <c r="I13" s="19">
+        <v>45.0</v>
+      </c>
+      <c r="J13" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="K13" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="L13" s="22">
+        <f t="shared" si="1"/>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="20">
+        <v>0.047</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G14" s="21">
+        <v>34.9</v>
+      </c>
+      <c r="H14" s="19">
+        <v>59.0</v>
+      </c>
+      <c r="I14" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="J14" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="K14" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="L14" s="22">
+        <f t="shared" si="1"/>
+        <v>47.25</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E15" s="20">
+        <v>0.06</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0.44</v>
+      </c>
+      <c r="G15" s="2">
+        <v>73.9</v>
+      </c>
+      <c r="H15" s="19">
+        <v>30.0</v>
+      </c>
+      <c r="I15" s="19">
+        <v>55.0</v>
+      </c>
+      <c r="J15" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="K15" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="L15" s="22">
+        <f t="shared" si="1"/>
+        <v>43.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" s="20">
+        <v>0.053</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0.44</v>
+      </c>
+      <c r="G16" s="21">
+        <v>69.9</v>
+      </c>
+      <c r="H16" s="19">
+        <v>70.0</v>
+      </c>
+      <c r="I16" s="19">
+        <v>30.0</v>
+      </c>
+      <c r="J16" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="K16" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="L16" s="22">
+        <f t="shared" si="1"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="E17" s="20"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="19"/>
+      <c r="L17" s="22"/>
+    </row>
+    <row r="18">
+      <c r="E18" s="20"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
+      <c r="L18" s="22"/>
+    </row>
+    <row r="19">
+      <c r="E19" s="20"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="L19" s="22"/>
+    </row>
+    <row r="20">
+      <c r="E20" s="20"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+      <c r="L20" s="22"/>
+    </row>
+    <row r="21">
+      <c r="E21" s="20"/>
+      <c r="G21" s="21"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="19"/>
+      <c r="L21" s="22"/>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update model 2025 (#3)
* train model for 2025 beers

* improve ux: constrain types, suggest breweries

* update metadata
</commit_message>
<xml_diff>
--- a/backend/Statistikk Juleøl.xlsx
+++ b/backend/Statistikk Juleøl.xlsx
@@ -7,25 +7,26 @@
     <sheet state="visible" name="2022" sheetId="2" r:id="rId5"/>
     <sheet state="visible" name="2023" sheetId="3" r:id="rId6"/>
     <sheet state="visible" name="2024" sheetId="4" r:id="rId7"/>
+    <sheet state="visible" name="2025" sheetId="5" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="1" name="Z_C71C843A_EAB5_42B1_B1FD_81E558391A10_.wvu.FilterData">'2022'!$A$1:$A$14</definedName>
-    <definedName hidden="1" localSheetId="2" name="Z_C71C843A_EAB5_42B1_B1FD_81E558391A10_.wvu.FilterData">'2023'!$A$1:$A$14</definedName>
-    <definedName hidden="1" localSheetId="0" name="Z_A5D866E3_0697_42C0_A55F_3D9EB20CFB23_.wvu.FilterData">'2020'!$J$1:$J$19</definedName>
-    <definedName hidden="1" localSheetId="1" name="Z_A5D866E3_0697_42C0_A55F_3D9EB20CFB23_.wvu.FilterData">'2022'!$A$2:$J$14</definedName>
-    <definedName hidden="1" localSheetId="2" name="Z_A5D866E3_0697_42C0_A55F_3D9EB20CFB23_.wvu.FilterData">'2023'!$A$2:$J$14</definedName>
-    <definedName hidden="1" localSheetId="3" name="Z_A5D866E3_0697_42C0_A55F_3D9EB20CFB23_.wvu.FilterData">'2024'!$B$2:$I$30</definedName>
+    <definedName hidden="1" localSheetId="1" name="Z_6393740B_0DC1_4FF3_81AB_78517B923F87_.wvu.FilterData">'2022'!$A$1:$A$14</definedName>
+    <definedName hidden="1" localSheetId="2" name="Z_6393740B_0DC1_4FF3_81AB_78517B923F87_.wvu.FilterData">'2023'!$A$1:$A$14</definedName>
+    <definedName hidden="1" localSheetId="0" name="Z_BE750BA2_1E5A_4896_A3E0_39DCEBB13DE6_.wvu.FilterData">'2020'!$J$1:$J$19</definedName>
+    <definedName hidden="1" localSheetId="1" name="Z_BE750BA2_1E5A_4896_A3E0_39DCEBB13DE6_.wvu.FilterData">'2022'!$A$2:$J$14</definedName>
+    <definedName hidden="1" localSheetId="2" name="Z_BE750BA2_1E5A_4896_A3E0_39DCEBB13DE6_.wvu.FilterData">'2023'!$A$2:$J$14</definedName>
+    <definedName hidden="1" localSheetId="3" name="Z_BE750BA2_1E5A_4896_A3E0_39DCEBB13DE6_.wvu.FilterData">'2024'!$B$2:$I$30</definedName>
   </definedNames>
   <calcPr/>
   <customWorkbookViews>
-    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{C71C843A-EAB5-42B1-B1FD-81E558391A10}" name="Filter 2"/>
-    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{A5D866E3-0697-42C0-A55F-3D9EB20CFB23}" name="Filter 1"/>
+    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{6393740B-0DC1-4FF3-81AB-78517B923F87}" name="Filter 2"/>
+    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{BE750BA2-1E5A-4896-A3E0-39DCEBB13DE6}" name="Filter 1"/>
   </customWorkbookViews>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="117">
   <si>
     <t>Nummer</t>
   </si>
@@ -138,9 +139,6 @@
     <t>Mack Juleøl</t>
   </si>
   <si>
-    <t>Macks Ølbryggeri</t>
-  </si>
-  <si>
     <t>Nordlandspils Juleøl</t>
   </si>
   <si>
@@ -193,6 +191,9 @@
   </si>
   <si>
     <t>IPA</t>
+  </si>
+  <si>
+    <t>Macks Ølbryggeri</t>
   </si>
   <si>
     <t>Gouden Carolus Christmas</t>
@@ -338,6 +339,45 @@
   <si>
     <t>Hansa Juleøl</t>
   </si>
+  <si>
+    <t>Flåklypa Spesial Juleøl</t>
+  </si>
+  <si>
+    <t>Nøisom</t>
+  </si>
+  <si>
+    <t>To Øl Jule Sovs Hazy IPA</t>
+  </si>
+  <si>
+    <t>Nøgne Ø Julequad</t>
+  </si>
+  <si>
+    <t>Ringnes Juleøl Sterk</t>
+  </si>
+  <si>
+    <t>Delirium</t>
+  </si>
+  <si>
+    <t>Cervisiam Santa Mental Sour Cream Pie</t>
+  </si>
+  <si>
+    <t>Cervisiam Bryggeri</t>
+  </si>
+  <si>
+    <t>Julekula 2025 Barrel Aged</t>
+  </si>
+  <si>
+    <t>Tuborg Juleøl Butikk</t>
+  </si>
+  <si>
+    <t>Gildeskål Saison</t>
+  </si>
+  <si>
+    <t>Bådin</t>
+  </si>
+  <si>
+    <t>Santas Break Red Lager</t>
+  </si>
 </sst>
 </file>
 
@@ -378,7 +418,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -427,6 +467,15 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -448,6 +497,10 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -1000,7 +1053,7 @@
         <v>36</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>27</v>
@@ -1027,10 +1080,10 @@
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="3"/>
       <c r="B13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>27</v>
@@ -1057,10 +1110,10 @@
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="3"/>
       <c r="B14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>27</v>
@@ -1087,13 +1140,13 @@
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="3"/>
       <c r="B15" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="8" t="s">
         <v>43</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>44</v>
       </c>
       <c r="E15" s="4">
         <v>0.06</v>
@@ -1117,10 +1170,10 @@
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="3"/>
       <c r="B16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>27</v>
@@ -1147,7 +1200,7 @@
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="3"/>
       <c r="B17" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>19</v>
@@ -1177,10 +1230,10 @@
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="3"/>
       <c r="B18" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>27</v>
@@ -1207,10 +1260,10 @@
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="3"/>
       <c r="B19" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>27</v>
@@ -1238,7 +1291,7 @@
     <row r="21" ht="15.75" customHeight="1"/>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{A5D866E3-0697-42C0-A55F-3D9EB20CFB23}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{BE750BA2-1E5A-4896-A3E0-39DCEBB13DE6}" filter="1" showAutoFilter="1">
       <autoFilter ref="$J$1:$J$19"/>
     </customSheetView>
   </customSheetViews>
@@ -1304,13 +1357,13 @@
         <v>11.0</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="E2" s="4">
         <v>0.06</v>
@@ -1338,13 +1391,13 @@
         <v>1.0</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="E3" s="4">
         <v>0.065</v>
@@ -1373,7 +1426,7 @@
         <v>36</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>27</v>
@@ -1608,10 +1661,10 @@
         <v>8.0</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>27</v>
@@ -9616,10 +9669,10 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{A5D866E3-0697-42C0-A55F-3D9EB20CFB23}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{BE750BA2-1E5A-4896-A3E0-39DCEBB13DE6}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$2:$J$14"/>
     </customSheetView>
-    <customSheetView guid="{C71C843A-EAB5-42B1-B1FD-81E558391A10}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{6393740B-0DC1-4FF3-81AB-78517B923F87}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$A$14">
         <filterColumn colId="0">
           <filters>
@@ -9701,13 +9754,13 @@
         <v>6.0</v>
       </c>
       <c r="B2" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>52</v>
       </c>
       <c r="E2" s="15">
         <v>0.06</v>
@@ -9776,7 +9829,7 @@
         <v>72</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>20</v>
@@ -9921,7 +9974,7 @@
         <v>16</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E8" s="15">
         <v>0.085</v>
@@ -9954,7 +10007,7 @@
         <v>36</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>27</v>
@@ -18021,10 +18074,10 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{A5D866E3-0697-42C0-A55F-3D9EB20CFB23}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{BE750BA2-1E5A-4896-A3E0-39DCEBB13DE6}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$2:$J$14"/>
     </customSheetView>
-    <customSheetView guid="{C71C843A-EAB5-42B1-B1FD-81E558391A10}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{6393740B-0DC1-4FF3-81AB-78517B923F87}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$A$14">
         <filterColumn colId="0">
           <filters>
@@ -18147,7 +18200,7 @@
         <v>84</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>20</v>
@@ -18339,13 +18392,13 @@
         <v>2.0</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="14" t="s">
         <v>51</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>52</v>
       </c>
       <c r="E8" s="15">
         <v>0.06</v>
@@ -18420,7 +18473,7 @@
         <v>93</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>20</v>
@@ -18501,7 +18554,7 @@
         <v>95</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E12" s="15">
         <v>0.074</v>
@@ -18579,7 +18632,7 @@
         <v>91</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E14" s="15">
         <v>0.06</v>
@@ -18618,7 +18671,7 @@
         <v>91</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E15" s="15">
         <v>0.065</v>
@@ -18654,7 +18707,7 @@
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>27</v>
@@ -18693,7 +18746,7 @@
         <v>100</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>27</v>
@@ -18732,7 +18785,7 @@
         <v>101</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>27</v>
@@ -18771,7 +18824,7 @@
         <v>102</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>27</v>
@@ -18846,10 +18899,10 @@
         <v>19.0</v>
       </c>
       <c r="B21" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>27</v>
@@ -24817,7 +24870,7 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{A5D866E3-0697-42C0-A55F-3D9EB20CFB23}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{BE750BA2-1E5A-4896-A3E0-39DCEBB13DE6}" filter="1" showAutoFilter="1">
       <autoFilter ref="$B$2:$I$30"/>
     </customSheetView>
   </customSheetViews>
@@ -24826,4 +24879,670 @@
   <pageSetup fitToHeight="0" paperSize="9" orientation="landscape" pageOrder="overThenDown"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <v>8.0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="20">
+        <v>0.06</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="G2" s="21">
+        <v>69.9</v>
+      </c>
+      <c r="H2" s="19">
+        <v>85.0</v>
+      </c>
+      <c r="I2" s="19">
+        <v>80.0</v>
+      </c>
+      <c r="J2" s="2">
+        <v>100.0</v>
+      </c>
+      <c r="K2" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="L2" s="22">
+        <f t="shared" ref="L2:L16" si="1">AVERAGE(H2:K2)</f>
+        <v>84.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" s="20">
+        <v>0.06</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="G3" s="21">
+        <v>159.9</v>
+      </c>
+      <c r="H3" s="19">
+        <v>87.0</v>
+      </c>
+      <c r="I3" s="19">
+        <v>75.0</v>
+      </c>
+      <c r="J3" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="K3" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="L3" s="22">
+        <f t="shared" si="1"/>
+        <v>75.75</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>9.0</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="20">
+        <v>0.102</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G4" s="21">
+        <v>138.0</v>
+      </c>
+      <c r="H4" s="19">
+        <v>74.0</v>
+      </c>
+      <c r="I4" s="19">
+        <v>67.0</v>
+      </c>
+      <c r="J4" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="K4" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="L4" s="22">
+        <f t="shared" si="1"/>
+        <v>68.25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>10.0</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" s="20">
+        <v>0.061</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.44</v>
+      </c>
+      <c r="G5" s="21">
+        <v>91.9</v>
+      </c>
+      <c r="H5" s="19">
+        <v>72.0</v>
+      </c>
+      <c r="I5" s="19">
+        <v>65.0</v>
+      </c>
+      <c r="J5" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="K5" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="L5" s="22">
+        <f t="shared" si="1"/>
+        <v>66.75</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>12.0</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="20">
+        <v>0.065</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="G6" s="2">
+        <v>49.9</v>
+      </c>
+      <c r="H6" s="19">
+        <v>82.0</v>
+      </c>
+      <c r="I6" s="19">
+        <v>60.0</v>
+      </c>
+      <c r="J6" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="K6" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="L6" s="22">
+        <f t="shared" si="1"/>
+        <v>66.75</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="20">
+        <v>0.09</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="G7" s="2">
+        <v>50.1</v>
+      </c>
+      <c r="H7" s="19">
+        <v>55.0</v>
+      </c>
+      <c r="I7" s="19">
+        <v>68.0</v>
+      </c>
+      <c r="J7" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="K7" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="L7" s="22">
+        <f t="shared" si="1"/>
+        <v>61.75</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>13.0</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" s="20">
+        <v>0.12</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G8" s="2">
+        <v>89.9</v>
+      </c>
+      <c r="H8" s="19">
+        <v>50.0</v>
+      </c>
+      <c r="I8" s="19">
+        <v>70.0</v>
+      </c>
+      <c r="J8" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="K8" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="L8" s="22">
+        <f t="shared" si="1"/>
+        <v>59.25</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="20">
+        <v>0.063</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="G9" s="21">
+        <v>41.9</v>
+      </c>
+      <c r="H9" s="19">
+        <v>65.0</v>
+      </c>
+      <c r="I9" s="19">
+        <v>50.0</v>
+      </c>
+      <c r="J9" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="K9" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="L9" s="22">
+        <f t="shared" si="1"/>
+        <v>58.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="20">
+        <v>0.06</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="G10" s="21">
+        <v>44.9</v>
+      </c>
+      <c r="H10" s="19">
+        <v>75.0</v>
+      </c>
+      <c r="I10" s="19">
+        <v>66.0</v>
+      </c>
+      <c r="J10" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="K10" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="L10" s="22">
+        <f t="shared" si="1"/>
+        <v>57.75</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2">
+        <v>7.0</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="20">
+        <v>0.1</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="G11" s="21">
+        <v>159.9</v>
+      </c>
+      <c r="H11" s="19">
+        <v>76.0</v>
+      </c>
+      <c r="I11" s="19">
+        <v>25.0</v>
+      </c>
+      <c r="J11" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="K11" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="L11" s="22">
+        <f t="shared" si="1"/>
+        <v>56.75</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="20">
+        <v>0.057</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="G12" s="21">
+        <v>90.4</v>
+      </c>
+      <c r="H12" s="19">
+        <v>55.0</v>
+      </c>
+      <c r="I12" s="19">
+        <v>69.0</v>
+      </c>
+      <c r="J12" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="K12" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="L12" s="22">
+        <f t="shared" si="1"/>
+        <v>56.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2">
+        <v>11.0</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="20">
+        <v>0.08</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.44</v>
+      </c>
+      <c r="G13" s="21">
+        <v>120.2</v>
+      </c>
+      <c r="H13" s="19">
+        <v>62.0</v>
+      </c>
+      <c r="I13" s="19">
+        <v>45.0</v>
+      </c>
+      <c r="J13" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="K13" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="L13" s="22">
+        <f t="shared" si="1"/>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="20">
+        <v>0.047</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G14" s="21">
+        <v>34.9</v>
+      </c>
+      <c r="H14" s="19">
+        <v>59.0</v>
+      </c>
+      <c r="I14" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="J14" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="K14" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="L14" s="22">
+        <f t="shared" si="1"/>
+        <v>47.25</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E15" s="20">
+        <v>0.06</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0.44</v>
+      </c>
+      <c r="G15" s="2">
+        <v>73.9</v>
+      </c>
+      <c r="H15" s="19">
+        <v>30.0</v>
+      </c>
+      <c r="I15" s="19">
+        <v>55.0</v>
+      </c>
+      <c r="J15" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="K15" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="L15" s="22">
+        <f t="shared" si="1"/>
+        <v>43.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" s="20">
+        <v>0.053</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0.44</v>
+      </c>
+      <c r="G16" s="21">
+        <v>69.9</v>
+      </c>
+      <c r="H16" s="19">
+        <v>70.0</v>
+      </c>
+      <c r="I16" s="19">
+        <v>30.0</v>
+      </c>
+      <c r="J16" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="K16" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="L16" s="22">
+        <f t="shared" si="1"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="E17" s="20"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="19"/>
+      <c r="L17" s="22"/>
+    </row>
+    <row r="18">
+      <c r="E18" s="20"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
+      <c r="L18" s="22"/>
+    </row>
+    <row r="19">
+      <c r="E19" s="20"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="L19" s="22"/>
+    </row>
+    <row r="20">
+      <c r="E20" s="20"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+      <c r="L20" s="22"/>
+    </row>
+    <row r="21">
+      <c r="E21" s="20"/>
+      <c r="G21" s="21"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="19"/>
+      <c r="L21" s="22"/>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>